<commit_message>
Update survival gameplay and balancing
</commit_message>
<xml_diff>
--- a/public/game-data/Lantern-Survival-Game-Config.xlsx
+++ b/public/game-data/Lantern-Survival-Game-Config.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4d4130e206d74b64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="2" r:id="Rb12323d35a564a06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="3" r:id="Rcfc8be20794c463f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="Rb1f7357fb6e24f09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="5" r:id="R5f7e985b8b7f4b24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R904ae0aea0af421d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfb91132757594819"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="2" r:id="Rf67544daeb064c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="3" r:id="Raa361ce686c54774"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="R014184d5004c4c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="5" r:id="R3f33594f79a743ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R503c0163dd404ab6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -366,7 +366,7 @@
         <x:v>新增怪物</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>Enemies 工作表新增一列；behavior 先使用 melee 或 ranged。</x:v>
+        <x:v>Enemies 工作表新增一列；behavior 可使用 melee、ranged 或 dashRetreat。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -402,7 +402,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="30.6299991607666" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="31.75" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="5.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="3.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="20.75" hidden="0" customWidth="1"/>
@@ -517,10 +517,10 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>player.moveSpeed.decayPerSecond</x:v>
+        <x:v>player.moveSpeed.maximum</x:v>
       </x:c>
       <x:c r="B11" s="12" t="n">
-        <x:v>1.4</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str"/>
       <x:c r="D11" s="12" t="str">
@@ -529,10 +529,10 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>lantern.radius.start</x:v>
+        <x:v>player.moveSpeed.decayPerSecond</x:v>
       </x:c>
       <x:c r="B12" s="12" t="n">
-        <x:v>210</x:v>
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str"/>
       <x:c r="D12" s="12" t="str">
@@ -541,10 +541,10 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>lantern.radius.minimum</x:v>
+        <x:v>player.color.darkenPerSecond</x:v>
       </x:c>
       <x:c r="B13" s="12" t="n">
-        <x:v>75</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str"/>
       <x:c r="D13" s="12" t="str">
@@ -553,10 +553,10 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>lantern.radius.decayPerSecond</x:v>
+        <x:v>player.color.restorePerSecond</x:v>
       </x:c>
       <x:c r="B14" s="12" t="n">
-        <x:v>1.05</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str"/>
       <x:c r="D14" s="12" t="str">
@@ -565,10 +565,10 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>lightDamage.dps.start</x:v>
+        <x:v>player.color.minimumBrightness</x:v>
       </x:c>
       <x:c r="B15" s="12" t="n">
-        <x:v>28</x:v>
+        <x:v>0.08</x:v>
       </x:c>
       <x:c r="C15" s="12" t="str"/>
       <x:c r="D15" s="12" t="str">
@@ -577,10 +577,10 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>lightDamage.dps.minimum</x:v>
+        <x:v>lantern.radius.start</x:v>
       </x:c>
       <x:c r="B16" s="12" t="n">
-        <x:v>5</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str"/>
       <x:c r="D16" s="12" t="str">
@@ -589,10 +589,10 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>lightDamage.dps.decayPerSecond</x:v>
+        <x:v>lantern.radius.minimum</x:v>
       </x:c>
       <x:c r="B17" s="12" t="n">
-        <x:v>0.18</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str"/>
       <x:c r="D17" s="12" t="str">
@@ -601,10 +601,10 @@
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>damageReduction.ratio.start</x:v>
+        <x:v>lantern.radius.maximum</x:v>
       </x:c>
       <x:c r="B18" s="12" t="n">
-        <x:v>0.55</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str"/>
       <x:c r="D18" s="12" t="str">
@@ -613,10 +613,10 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>damageReduction.ratio.minimum</x:v>
+        <x:v>lantern.radius.decayPerSecond</x:v>
       </x:c>
       <x:c r="B19" s="12" t="n">
-        <x:v>0.08</x:v>
+        <x:v>1.05</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str"/>
       <x:c r="D19" s="12" t="str">
@@ -625,10 +625,10 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
-        <x:v>damageReduction.ratio.decayPerSecond</x:v>
+        <x:v>lightDamage.dps.start</x:v>
       </x:c>
       <x:c r="B20" s="12" t="n">
-        <x:v>0.004</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C20" s="12" t="str"/>
       <x:c r="D20" s="12" t="str">
@@ -637,10 +637,10 @@
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>healthDrain.startPerSecond</x:v>
+        <x:v>lightDamage.dps.minimum</x:v>
       </x:c>
       <x:c r="B21" s="12" t="n">
-        <x:v>0.8</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C21" s="12" t="str"/>
       <x:c r="D21" s="12" t="str">
@@ -649,10 +649,10 @@
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
-        <x:v>healthDrain.increasePerSecond</x:v>
+        <x:v>lightDamage.dps.maximum</x:v>
       </x:c>
       <x:c r="B22" s="12" t="n">
-        <x:v>0.035</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C22" s="12" t="str"/>
       <x:c r="D22" s="12" t="str">
@@ -661,10 +661,10 @@
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="12" t="str">
-        <x:v>healthDrain.curve</x:v>
-      </x:c>
-      <x:c r="B23" s="12" t="str">
-        <x:v>linear</x:v>
+        <x:v>lightDamage.dps.decayPerSecond</x:v>
+      </x:c>
+      <x:c r="B23" s="12" t="n">
+        <x:v>0.18</x:v>
       </x:c>
       <x:c r="C23" s="12" t="str"/>
       <x:c r="D23" s="12" t="str">
@@ -673,10 +673,10 @@
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>healthDrain.quadraticFactor</x:v>
+        <x:v>damageReduction.ratio.start</x:v>
       </x:c>
       <x:c r="B24" s="12" t="n">
-        <x:v>0.0007</x:v>
+        <x:v>0.55</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str"/>
       <x:c r="D24" s="12" t="str">
@@ -685,10 +685,10 @@
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="12" t="str">
-        <x:v>pickups.spawnInterval</x:v>
+        <x:v>damageReduction.ratio.minimum</x:v>
       </x:c>
       <x:c r="B25" s="12" t="n">
-        <x:v>8</x:v>
+        <x:v>0.08</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str"/>
       <x:c r="D25" s="12" t="str">
@@ -697,10 +697,10 @@
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="12" t="str">
-        <x:v>pickups.lifetime</x:v>
+        <x:v>damageReduction.ratio.maximum</x:v>
       </x:c>
       <x:c r="B26" s="12" t="n">
-        <x:v>14</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="C26" s="12" t="str"/>
       <x:c r="D26" s="12" t="str">
@@ -709,10 +709,10 @@
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="12" t="str">
-        <x:v>pickups.pickupRange</x:v>
+        <x:v>damageReduction.ratio.decayPerSecond</x:v>
       </x:c>
       <x:c r="B27" s="12" t="n">
-        <x:v>34</x:v>
+        <x:v>0.004</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str"/>
       <x:c r="D27" s="12" t="str">
@@ -721,10 +721,10 @@
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="12" t="str">
-        <x:v>pickups.sharedHealthDrainReduction</x:v>
+        <x:v>healthDrain.startPerSecond</x:v>
       </x:c>
       <x:c r="B28" s="12" t="n">
-        <x:v>0.5</x:v>
+        <x:v>-1.2</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str"/>
       <x:c r="D28" s="12" t="str">
@@ -733,10 +733,10 @@
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="12" t="str">
-        <x:v>pickups.sharedEffectDuration</x:v>
+        <x:v>healthDrain.increasePerSecond</x:v>
       </x:c>
       <x:c r="B29" s="12" t="n">
-        <x:v>5</x:v>
+        <x:v>0.03</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str"/>
       <x:c r="D29" s="12" t="str">
@@ -745,10 +745,10 @@
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="12" t="str">
-        <x:v>enemies.spawnInterval</x:v>
+        <x:v>healthDrain.ageMultiplierScale</x:v>
       </x:c>
       <x:c r="B30" s="12" t="n">
-        <x:v>2.2</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str"/>
       <x:c r="D30" s="12" t="str">
@@ -757,10 +757,10 @@
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="12" t="str">
-        <x:v>enemies.minimumSpawnInterval</x:v>
-      </x:c>
-      <x:c r="B31" s="12" t="n">
-        <x:v>0.55</x:v>
+        <x:v>healthDrain.curve</x:v>
+      </x:c>
+      <x:c r="B31" s="12" t="str">
+        <x:v>linear</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str"/>
       <x:c r="D31" s="12" t="str">
@@ -769,10 +769,10 @@
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="12" t="str">
-        <x:v>enemies.spawnIntervalDecayPerSecond</x:v>
+        <x:v>healthDrain.quadraticFactor</x:v>
       </x:c>
       <x:c r="B32" s="12" t="n">
-        <x:v>0.012</x:v>
+        <x:v>0.0007</x:v>
       </x:c>
       <x:c r="C32" s="12" t="str"/>
       <x:c r="D32" s="12" t="str">
@@ -781,10 +781,10 @@
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="12" t="str">
-        <x:v>enemies.countStart</x:v>
+        <x:v>age.secondsPerYear</x:v>
       </x:c>
       <x:c r="B33" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C33" s="12" t="str"/>
       <x:c r="D33" s="12" t="str">
@@ -793,10 +793,10 @@
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="12" t="str">
-        <x:v>enemies.countIncreaseEverySeconds</x:v>
+        <x:v>age.slowStart</x:v>
       </x:c>
       <x:c r="B34" s="12" t="n">
-        <x:v>35</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str"/>
       <x:c r="D34" s="12" t="str">
@@ -805,10 +805,10 @@
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="12" t="str">
-        <x:v>enemies.countMaximum</x:v>
+        <x:v>age.mediumStart</x:v>
       </x:c>
       <x:c r="B35" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C35" s="12" t="str"/>
       <x:c r="D35" s="12" t="str">
@@ -817,10 +817,10 @@
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="12" t="str">
-        <x:v>projectile.lifetime</x:v>
+        <x:v>age.fastStart</x:v>
       </x:c>
       <x:c r="B36" s="12" t="n">
-        <x:v>5</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C36" s="12" t="str"/>
       <x:c r="D36" s="12" t="str">
@@ -829,13 +829,217 @@
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
-        <x:v>projectile.radius</x:v>
+        <x:v>age.slowMultiplier</x:v>
       </x:c>
       <x:c r="B37" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="C37" s="12" t="str"/>
       <x:c r="D37" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="A38" s="12" t="str">
+        <x:v>age.mediumMultiplier</x:v>
+      </x:c>
+      <x:c r="B38" s="12" t="n">
+        <x:v>1.7</x:v>
+      </x:c>
+      <x:c r="C38" s="12" t="str"/>
+      <x:c r="D38" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="A39" s="12" t="str">
+        <x:v>age.fastMultiplier</x:v>
+      </x:c>
+      <x:c r="B39" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C39" s="12" t="str"/>
+      <x:c r="D39" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
+      <x:c r="A40" s="12" t="str">
+        <x:v>pickups.spawnInterval</x:v>
+      </x:c>
+      <x:c r="B40" s="12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C40" s="12" t="str"/>
+      <x:c r="D40" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="15" hidden="0" customHeight="1">
+      <x:c r="A41" s="12" t="str">
+        <x:v>pickups.lifetime</x:v>
+      </x:c>
+      <x:c r="B41" s="12" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C41" s="12" t="str"/>
+      <x:c r="D41" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="12" t="str">
+        <x:v>pickups.pickupRange</x:v>
+      </x:c>
+      <x:c r="B42" s="12" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="C42" s="12" t="str"/>
+      <x:c r="D42" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="12" t="str">
+        <x:v>pickups.sharedHealthDrainReduction</x:v>
+      </x:c>
+      <x:c r="B43" s="12" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C43" s="12" t="str"/>
+      <x:c r="D43" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="12" t="str">
+        <x:v>pickups.sharedEffectDuration</x:v>
+      </x:c>
+      <x:c r="B44" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C44" s="12" t="str"/>
+      <x:c r="D44" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="12" t="str">
+        <x:v>enemies.spawnInterval</x:v>
+      </x:c>
+      <x:c r="B45" s="12" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="C45" s="12" t="str"/>
+      <x:c r="D45" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="12" t="str">
+        <x:v>enemies.earlyAgeSpawnIntervalMultiplier</x:v>
+      </x:c>
+      <x:c r="B46" s="12" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="C46" s="12" t="str"/>
+      <x:c r="D46" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
+      <x:c r="A47" s="12" t="str">
+        <x:v>enemies.minimumSpawnInterval</x:v>
+      </x:c>
+      <x:c r="B47" s="12" t="n">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="C47" s="12" t="str"/>
+      <x:c r="D47" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="A48" s="12" t="str">
+        <x:v>enemies.spawnIntervalDecayPerSecond</x:v>
+      </x:c>
+      <x:c r="B48" s="12" t="n">
+        <x:v>0.0035</x:v>
+      </x:c>
+      <x:c r="C48" s="12" t="str"/>
+      <x:c r="D48" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="A49" s="12" t="str">
+        <x:v>enemies.countStart</x:v>
+      </x:c>
+      <x:c r="B49" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C49" s="12" t="str"/>
+      <x:c r="D49" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="A50" s="12" t="str">
+        <x:v>enemies.countIncreaseAmount</x:v>
+      </x:c>
+      <x:c r="B50" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C50" s="12" t="str"/>
+      <x:c r="D50" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="A51" s="12" t="str">
+        <x:v>enemies.countIncreaseEverySeconds</x:v>
+      </x:c>
+      <x:c r="B51" s="12" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="C51" s="12" t="str"/>
+      <x:c r="D51" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="12" t="str">
+        <x:v>enemies.countMaximum</x:v>
+      </x:c>
+      <x:c r="B52" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C52" s="12" t="str"/>
+      <x:c r="D52" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="12" t="str">
+        <x:v>projectile.lifetime</x:v>
+      </x:c>
+      <x:c r="B53" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C53" s="12" t="str"/>
+      <x:c r="D53" s="12" t="str">
+        <x:v>在這裡調整遊戲平衡數值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="12" t="str">
+        <x:v>projectile.radius</x:v>
+      </x:c>
+      <x:c r="B54" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C54" s="12" t="str"/>
+      <x:c r="D54" s="12" t="str">
         <x:v>在這裡調整遊戲平衡數值</x:v>
       </x:c>
     </x:row>
@@ -858,10 +1062,18 @@
     <x:col min="8" max="8" width="14.5" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="5.130000114440918" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="14.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="11.130000114440918" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="11.130000114440918" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="7.5" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12.75" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12.75" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="9.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="11.25" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="10.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="9.5" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="14.5" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="10.75" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="12.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="10.5" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="20.6299991607666" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="12.380000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -881,6 +1093,14 @@
       <x:c r="L1" s="7"/>
       <x:c r="M1" s="7"/>
       <x:c r="N1" s="7"/>
+      <x:c r="O1" s="7"/>
+      <x:c r="P1" s="7"/>
+      <x:c r="Q1" s="7"/>
+      <x:c r="R1" s="7"/>
+      <x:c r="S1" s="7"/>
+      <x:c r="T1" s="7"/>
+      <x:c r="U1" s="7"/>
+      <x:c r="V1" s="7"/>
     </x:row>
     <x:row r="2"/>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -926,6 +1146,30 @@
       <x:c r="N3" s="10" t="str">
         <x:v>spawnWeight</x:v>
       </x:c>
+      <x:c r="O3" s="10" t="str">
+        <x:v>triggerRange</x:v>
+      </x:c>
+      <x:c r="P3" s="10" t="str">
+        <x:v>dashSpeed</x:v>
+      </x:c>
+      <x:c r="Q3" s="10" t="str">
+        <x:v>dashEndDistance</x:v>
+      </x:c>
+      <x:c r="R3" s="10" t="str">
+        <x:v>retreatSpeed</x:v>
+      </x:c>
+      <x:c r="S3" s="10" t="str">
+        <x:v>retreatDuration</x:v>
+      </x:c>
+      <x:c r="T3" s="10" t="str">
+        <x:v>statusEffect</x:v>
+      </x:c>
+      <x:c r="U3" s="10" t="str">
+        <x:v>statusDamagePerSecond</x:v>
+      </x:c>
+      <x:c r="V3" s="10" t="str">
+        <x:v>statusDuration</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -968,8 +1212,16 @@
         <x:v>melee</x:v>
       </x:c>
       <x:c r="N4" s="12" t="n">
-        <x:v>0.68</x:v>
-      </x:c>
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="O4" s="12" t="str"/>
+      <x:c r="P4" s="12" t="str"/>
+      <x:c r="Q4" s="12" t="str"/>
+      <x:c r="R4" s="12" t="str"/>
+      <x:c r="S4" s="12" t="str"/>
+      <x:c r="T4" s="12" t="str"/>
+      <x:c r="U4" s="12" t="str"/>
+      <x:c r="V4" s="12" t="str"/>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
@@ -1012,7 +1264,83 @@
         <x:v>ranged</x:v>
       </x:c>
       <x:c r="N5" s="12" t="n">
-        <x:v>0.32</x:v>
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="O5" s="12" t="str"/>
+      <x:c r="P5" s="12" t="str"/>
+      <x:c r="Q5" s="12" t="str"/>
+      <x:c r="R5" s="12" t="str"/>
+      <x:c r="S5" s="12" t="str"/>
+      <x:c r="T5" s="12" t="str"/>
+      <x:c r="U5" s="12" t="str"/>
+      <x:c r="V5" s="12" t="str"/>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="12" t="str">
+        <x:v>mosquito</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>蚊子</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="E6" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F6" s="12" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="G6" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H6" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I6" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J6" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K6" s="12" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="L6" s="12" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="M6" s="12" t="str">
+        <x:v>dashRetreat</x:v>
+      </x:c>
+      <x:c r="N6" s="12" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="O6" s="12" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="P6" s="12" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="Q6" s="12" t="n">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="R6" s="12" t="n">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="S6" s="12" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="T6" s="12" t="str">
+        <x:v>mosquitoBite</x:v>
+      </x:c>
+      <x:c r="U6" s="12" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="V6" s="12" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1426,6 +1754,110 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="12" t="str">
+        <x:v>player</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="str">
+        <x:v>hurtUp</x:v>
+      </x:c>
+      <x:c r="C12" s="12" t="str">
+        <x:v>player_hurt_up</x:v>
+      </x:c>
+      <x:c r="D12" s="12" t="str">
+        <x:v>player</x:v>
+      </x:c>
+      <x:c r="E12" s="12" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F12" s="12" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="G12" s="12" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H12" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="12" t="str">
+        <x:v>player</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="str">
+        <x:v>hurtSide</x:v>
+      </x:c>
+      <x:c r="C13" s="12" t="str">
+        <x:v>player_hurt_side</x:v>
+      </x:c>
+      <x:c r="D13" s="12" t="str">
+        <x:v>player</x:v>
+      </x:c>
+      <x:c r="E13" s="12" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F13" s="12" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="G13" s="12" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H13" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="12" t="str">
+        <x:v>player</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>deathUp</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="str">
+        <x:v>player_death_up</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="str">
+        <x:v>player</x:v>
+      </x:c>
+      <x:c r="E14" s="12" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="F14" s="12" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="G14" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H14" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="12" t="str">
+        <x:v>player</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="str">
+        <x:v>deathSide</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="str">
+        <x:v>player_death_side</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="str">
+        <x:v>player</x:v>
+      </x:c>
+      <x:c r="E15" s="12" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="F15" s="12" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="G15" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H15" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1436,7 +1868,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="22.25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="11.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.75" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="23.5" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="9.75" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="10.25" hidden="0" customWidth="1"/>
@@ -1622,10 +2054,10 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>projectile</x:v>
+        <x:v>enemyMosquito</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>projectile</x:v>
+        <x:v>enemyMosquito</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str"/>
       <x:c r="D7" s="12" t="str"/>
@@ -1640,27 +2072,27 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="I7" s="12" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J7" s="12" t="str">
-        <x:v>circle</x:v>
+        <x:v>triangle</x:v>
       </x:c>
       <x:c r="K7" s="12" t="n">
-        <x:v>16741848</x:v>
+        <x:v>16743324</x:v>
       </x:c>
       <x:c r="L7" s="12" t="n">
-        <x:v>12</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="M7" s="12" t="n">
-        <x:v>12</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>pickupLight</x:v>
+        <x:v>projectile</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>pickupLight</x:v>
+        <x:v>projectile</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str"/>
       <x:c r="D8" s="12" t="str"/>
@@ -1675,29 +2107,31 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="I8" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J8" s="12" t="str">
         <x:v>circle</x:v>
       </x:c>
       <x:c r="K8" s="12" t="n">
-        <x:v>16766202</x:v>
+        <x:v>16741848</x:v>
       </x:c>
       <x:c r="L8" s="12" t="n">
-        <x:v>24</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="M8" s="12" t="n">
-        <x:v>24</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>pickupSpeed</x:v>
+        <x:v>pickupLight</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>pickupSpeed</x:v>
-      </x:c>
-      <x:c r="C9" s="12" t="str"/>
+        <x:v>pickupLight</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="str">
+        <x:v>assets/items/light-radius.png</x:v>
+      </x:c>
       <x:c r="D9" s="12" t="str"/>
       <x:c r="E9" s="12" t="str"/>
       <x:c r="F9" s="12" t="n">
@@ -1713,24 +2147,24 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J9" s="12" t="str">
-        <x:v>triangle</x:v>
+        <x:v>circle</x:v>
       </x:c>
       <x:c r="K9" s="12" t="n">
-        <x:v>4848817</x:v>
+        <x:v>16766202</x:v>
       </x:c>
       <x:c r="L9" s="12" t="n">
-        <x:v>26</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="M9" s="12" t="n">
-        <x:v>26</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
-        <x:v>pickupDamage</x:v>
+        <x:v>pickupSpeed</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>pickupDamage</x:v>
+        <x:v>pickupSpeed</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str"/>
       <x:c r="D10" s="12" t="str"/>
@@ -1748,24 +2182,24 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J10" s="12" t="str">
-        <x:v>rect</x:v>
+        <x:v>triangle</x:v>
       </x:c>
       <x:c r="K10" s="12" t="n">
-        <x:v>16747586</x:v>
+        <x:v>4848817</x:v>
       </x:c>
       <x:c r="L10" s="12" t="n">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="M10" s="12" t="n">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>pickupDefense</x:v>
+        <x:v>pickupDamage</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>pickupDefense</x:v>
+        <x:v>pickupDamage</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str"/>
       <x:c r="D11" s="12" t="str"/>
@@ -1786,12 +2220,47 @@
         <x:v>rect</x:v>
       </x:c>
       <x:c r="K11" s="12" t="n">
-        <x:v>5617407</x:v>
+        <x:v>16747586</x:v>
       </x:c>
       <x:c r="L11" s="12" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="M11" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="12" t="str">
+        <x:v>pickupDefense</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="str">
+        <x:v>pickupDefense</x:v>
+      </x:c>
+      <x:c r="C12" s="12" t="str"/>
+      <x:c r="D12" s="12" t="str"/>
+      <x:c r="E12" s="12" t="str"/>
+      <x:c r="F12" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G12" s="12" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H12" s="12" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="I12" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J12" s="12" t="str">
+        <x:v>rect</x:v>
+      </x:c>
+      <x:c r="K12" s="12" t="n">
+        <x:v>5617407</x:v>
+      </x:c>
+      <x:c r="L12" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M12" s="12" t="n">
         <x:v>24</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Integrate enemy animations and game assets
</commit_message>
<xml_diff>
--- a/public/game-data/Lantern-Survival-Game-Config.xlsx
+++ b/public/game-data/Lantern-Survival-Game-Config.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfb91132757594819"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="2" r:id="Rf67544daeb064c64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="3" r:id="Raa361ce686c54774"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="R014184d5004c4c4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="5" r:id="R3f33594f79a743ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R503c0163dd404ab6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1ab79b10e7e346a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="2" r:id="Re336613eaf4d46e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="3" r:id="R02b87ad10ab24ba2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="Rd5fb11f64e264bac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="5" r:id="Ra4ffb080a6b64412"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R75e5702accd04c1b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -53,7 +53,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -75,6 +75,21 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -82,7 +97,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -103,6 +118,19 @@
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1353,12 +1381,13 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="20.6299991607666" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="4.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="6" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="11.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="4.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="23.5" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="11.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11.130000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -1371,6 +1400,7 @@
       <x:c r="E1" s="7"/>
       <x:c r="F1" s="7"/>
       <x:c r="G1" s="7"/>
+      <x:c r="H1" s="7"/>
     </x:row>
     <x:row r="2"/>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -1395,6 +1425,9 @@
       <x:c r="G3" s="10" t="str">
         <x:v>effectDuration</x:v>
       </x:c>
+      <x:c r="H3" s="10" t="str">
+        <x:v>minimumAge</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -1418,6 +1451,7 @@
       <x:c r="G4" s="12" t="n">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="H4" s="12" t="str"/>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
@@ -1441,6 +1475,7 @@
       <x:c r="G5" s="12" t="n">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="H5" s="12" t="str"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
@@ -1464,6 +1499,7 @@
       <x:c r="G6" s="12" t="n">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="H6" s="12" t="str"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
@@ -1486,6 +1522,33 @@
       </x:c>
       <x:c r="G7" s="12" t="n">
         <x:v>5</x:v>
+      </x:c>
+      <x:c r="H7" s="12" t="str"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="12" t="str">
+        <x:v>youthFruit</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="str">
+        <x:v>青春果</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="str">
+        <x:v>pickupAge</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="str">
+        <x:v>ageReduction</x:v>
+      </x:c>
+      <x:c r="E8" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F8" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G8" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="12" t="n">
+        <x:v>35</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1497,14 +1560,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="27.25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="8.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="6.130000114440918" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="9.130000114440918" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="8.5" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="8.75" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="5.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -1855,6 +1918,396 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="H15" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="21" customHeight="1">
+      <x:c r="A16" s="17" t="str">
+        <x:v>enemyMelee</x:v>
+      </x:c>
+      <x:c r="B16" s="17" t="str">
+        <x:v>idle</x:v>
+      </x:c>
+      <x:c r="C16" s="17" t="str">
+        <x:v>melee_idle</x:v>
+      </x:c>
+      <x:c r="D16" s="17" t="str">
+        <x:v>enemyMelee</x:v>
+      </x:c>
+      <x:c r="E16" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G16" s="17" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H16" s="17" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="21" customHeight="1">
+      <x:c r="A17" s="17" t="str">
+        <x:v>enemyMelee</x:v>
+      </x:c>
+      <x:c r="B17" s="17" t="str">
+        <x:v>move</x:v>
+      </x:c>
+      <x:c r="C17" s="17" t="str">
+        <x:v>melee_move</x:v>
+      </x:c>
+      <x:c r="D17" s="17" t="str">
+        <x:v>enemyMelee</x:v>
+      </x:c>
+      <x:c r="E17" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="17" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G17" s="17" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H17" s="17" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="21" customHeight="1">
+      <x:c r="A18" s="17" t="str">
+        <x:v>enemyMelee</x:v>
+      </x:c>
+      <x:c r="B18" s="17" t="str">
+        <x:v>attack</x:v>
+      </x:c>
+      <x:c r="C18" s="17" t="str">
+        <x:v>melee_attack</x:v>
+      </x:c>
+      <x:c r="D18" s="17" t="str">
+        <x:v>enemyMelee</x:v>
+      </x:c>
+      <x:c r="E18" s="17" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F18" s="17" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G18" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H18" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="21" customHeight="1">
+      <x:c r="A19" s="17" t="str">
+        <x:v>enemyMelee</x:v>
+      </x:c>
+      <x:c r="B19" s="17" t="str">
+        <x:v>hurt</x:v>
+      </x:c>
+      <x:c r="C19" s="17" t="str">
+        <x:v>melee_hurt</x:v>
+      </x:c>
+      <x:c r="D19" s="17" t="str">
+        <x:v>enemyMelee</x:v>
+      </x:c>
+      <x:c r="E19" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F19" s="17" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G19" s="17" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H19" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="21" customHeight="1">
+      <x:c r="A20" s="17" t="str">
+        <x:v>enemyMelee</x:v>
+      </x:c>
+      <x:c r="B20" s="17" t="str">
+        <x:v>death</x:v>
+      </x:c>
+      <x:c r="C20" s="17" t="str">
+        <x:v>melee_death</x:v>
+      </x:c>
+      <x:c r="D20" s="17" t="str">
+        <x:v>enemyMelee</x:v>
+      </x:c>
+      <x:c r="E20" s="17" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F20" s="17" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G20" s="17" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H20" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="21" customHeight="1">
+      <x:c r="A21" s="17" t="str">
+        <x:v>enemyRanged</x:v>
+      </x:c>
+      <x:c r="B21" s="17" t="str">
+        <x:v>idle</x:v>
+      </x:c>
+      <x:c r="C21" s="17" t="str">
+        <x:v>ranged_idle</x:v>
+      </x:c>
+      <x:c r="D21" s="17" t="str">
+        <x:v>enemyRanged</x:v>
+      </x:c>
+      <x:c r="E21" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F21" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G21" s="17" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H21" s="17" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="21" customHeight="1">
+      <x:c r="A22" s="17" t="str">
+        <x:v>enemyRanged</x:v>
+      </x:c>
+      <x:c r="B22" s="17" t="str">
+        <x:v>move</x:v>
+      </x:c>
+      <x:c r="C22" s="17" t="str">
+        <x:v>ranged_move</x:v>
+      </x:c>
+      <x:c r="D22" s="17" t="str">
+        <x:v>enemyRanged</x:v>
+      </x:c>
+      <x:c r="E22" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F22" s="17" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G22" s="17" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H22" s="17" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="21" customHeight="1">
+      <x:c r="A23" s="17" t="str">
+        <x:v>enemyRanged</x:v>
+      </x:c>
+      <x:c r="B23" s="17" t="str">
+        <x:v>attack</x:v>
+      </x:c>
+      <x:c r="C23" s="17" t="str">
+        <x:v>ranged_attack</x:v>
+      </x:c>
+      <x:c r="D23" s="17" t="str">
+        <x:v>enemyRanged</x:v>
+      </x:c>
+      <x:c r="E23" s="17" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F23" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G23" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H23" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="21" customHeight="1">
+      <x:c r="A24" s="17" t="str">
+        <x:v>enemyRanged</x:v>
+      </x:c>
+      <x:c r="B24" s="17" t="str">
+        <x:v>hurt</x:v>
+      </x:c>
+      <x:c r="C24" s="17" t="str">
+        <x:v>ranged_hurt</x:v>
+      </x:c>
+      <x:c r="D24" s="17" t="str">
+        <x:v>enemyRanged</x:v>
+      </x:c>
+      <x:c r="E24" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F24" s="17" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G24" s="17" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H24" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="21" customHeight="1">
+      <x:c r="A25" s="17" t="str">
+        <x:v>enemyRanged</x:v>
+      </x:c>
+      <x:c r="B25" s="17" t="str">
+        <x:v>death</x:v>
+      </x:c>
+      <x:c r="C25" s="17" t="str">
+        <x:v>ranged_death</x:v>
+      </x:c>
+      <x:c r="D25" s="17" t="str">
+        <x:v>enemyRanged</x:v>
+      </x:c>
+      <x:c r="E25" s="17" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F25" s="17" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G25" s="17" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H25" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="21" customHeight="1">
+      <x:c r="A26" s="17" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="B26" s="17" t="str">
+        <x:v>idle</x:v>
+      </x:c>
+      <x:c r="C26" s="17" t="str">
+        <x:v>mosquito_idle</x:v>
+      </x:c>
+      <x:c r="D26" s="17" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="E26" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F26" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G26" s="17" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H26" s="17" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="21" customHeight="1">
+      <x:c r="A27" s="17" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="B27" s="17" t="str">
+        <x:v>move</x:v>
+      </x:c>
+      <x:c r="C27" s="17" t="str">
+        <x:v>mosquito_move</x:v>
+      </x:c>
+      <x:c r="D27" s="17" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="E27" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F27" s="17" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G27" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H27" s="17" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="21" customHeight="1">
+      <x:c r="A28" s="17" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="B28" s="17" t="str">
+        <x:v>attack</x:v>
+      </x:c>
+      <x:c r="C28" s="17" t="str">
+        <x:v>mosquito_attack</x:v>
+      </x:c>
+      <x:c r="D28" s="17" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="E28" s="17" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F28" s="17" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G28" s="17" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H28" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="21" customHeight="1">
+      <x:c r="A29" s="17" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="B29" s="17" t="str">
+        <x:v>hurt</x:v>
+      </x:c>
+      <x:c r="C29" s="17" t="str">
+        <x:v>mosquito_hurt</x:v>
+      </x:c>
+      <x:c r="D29" s="17" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="E29" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F29" s="17" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G29" s="17" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H29" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="21" customHeight="1">
+      <x:c r="A30" s="17" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="B30" s="17" t="str">
+        <x:v>death</x:v>
+      </x:c>
+      <x:c r="C30" s="17" t="str">
+        <x:v>mosquito_death</x:v>
+      </x:c>
+      <x:c r="D30" s="17" t="str">
+        <x:v>enemyMosquito</x:v>
+      </x:c>
+      <x:c r="E30" s="17" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F30" s="17" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G30" s="17" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H30" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1869,7 +2322,7 @@
   <x:cols>
     <x:col min="1" max="1" width="22.25" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12.75" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="23.5" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="9.75" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="10.25" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="4.75" hidden="0" customWidth="1"/>
@@ -1989,9 +2442,15 @@
       <x:c r="B5" s="12" t="str">
         <x:v>enemyMelee</x:v>
       </x:c>
-      <x:c r="C5" s="12" t="str"/>
-      <x:c r="D5" s="12" t="str"/>
-      <x:c r="E5" s="12" t="str"/>
+      <x:c r="C5" s="12" t="str">
+        <x:v>assets/enemies/enemy-melee-sheet.png</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
       <x:c r="F5" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -2024,9 +2483,15 @@
       <x:c r="B6" s="12" t="str">
         <x:v>enemyRanged</x:v>
       </x:c>
-      <x:c r="C6" s="12" t="str"/>
-      <x:c r="D6" s="12" t="str"/>
-      <x:c r="E6" s="12" t="str"/>
+      <x:c r="C6" s="12" t="str">
+        <x:v>assets/enemies/enemy-ranged-sheet.png</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E6" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
       <x:c r="F6" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -2059,9 +2524,15 @@
       <x:c r="B7" s="12" t="str">
         <x:v>enemyMosquito</x:v>
       </x:c>
-      <x:c r="C7" s="12" t="str"/>
-      <x:c r="D7" s="12" t="str"/>
-      <x:c r="E7" s="12" t="str"/>
+      <x:c r="C7" s="12" t="str">
+        <x:v>assets/enemies/enemy-mosquito-sheet.png</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E7" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
       <x:c r="F7" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -2264,6 +2735,41 @@
         <x:v>24</x:v>
       </x:c>
     </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="12" t="str">
+        <x:v>pickupAge</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="str">
+        <x:v>pickupAge</x:v>
+      </x:c>
+      <x:c r="C13" s="12" t="str"/>
+      <x:c r="D13" s="12" t="str"/>
+      <x:c r="E13" s="12" t="str"/>
+      <x:c r="F13" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G13" s="12" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H13" s="12" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="I13" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J13" s="12" t="str">
+        <x:v>circle</x:v>
+      </x:c>
+      <x:c r="K13" s="12" t="n">
+        <x:v>11958503</x:v>
+      </x:c>
+      <x:c r="L13" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M13" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add start screen and update game items
</commit_message>
<xml_diff>
--- a/public/game-data/Lantern-Survival-Game-Config.xlsx
+++ b/public/game-data/Lantern-Survival-Game-Config.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1ab79b10e7e346a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="2" r:id="Re336613eaf4d46e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="3" r:id="R02b87ad10ab24ba2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="Rd5fb11f64e264bac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="5" r:id="Ra4ffb080a6b64412"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R75e5702accd04c1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re6620ad47ed74b77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="2" r:id="R81909b72c6f448ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="3" r:id="R9fbeee63044a4b81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="Racdc5f85ef5641dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="5" r:id="R2e60fbe03ef34245"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Re4b140b2299f4b53"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -53,7 +53,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -90,6 +90,16 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -97,7 +107,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -132,11 +142,81 @@
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1365,10 +1445,10 @@
         <x:v>mosquitoBite</x:v>
       </x:c>
       <x:c r="U6" s="12" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="V6" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1383,11 +1463,13 @@
     <x:col min="1" max="1" width="20.6299991607666" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="6" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="11.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="4.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="23.5" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="11.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="11.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -1428,16 +1510,22 @@
       <x:c r="H3" s="10" t="str">
         <x:v>minimumAge</x:v>
       </x:c>
+      <x:c r="I3" s="22" t="str">
+        <x:v>ageReductionYears</x:v>
+      </x:c>
+      <x:c r="J3" s="22" t="str">
+        <x:v>clearsStatusEffects</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="12" t="str">
-        <x:v>lightBoost</x:v>
+        <x:v>nne</x:v>
       </x:c>
       <x:c r="B4" s="12" t="str">
-        <x:v>燈油</x:v>
+        <x:v>NNE</x:v>
       </x:c>
       <x:c r="C4" s="12" t="str">
-        <x:v>pickupLight</x:v>
+        <x:v>pickupNNE</x:v>
       </x:c>
       <x:c r="D4" s="12" t="str">
         <x:v>lightRadius</x:v>
@@ -1446,22 +1534,28 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="F4" s="12" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="12" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="H4" s="12" t="str"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H4" s="12"/>
+      <x:c r="I4" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J4" s="30" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>speedBoost</x:v>
+        <x:v>yss</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>疾風</x:v>
+        <x:v>YSS</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>pickupSpeed</x:v>
+        <x:v>pickupYSS</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
         <x:v>moveSpeed</x:v>
@@ -1470,52 +1564,64 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="F5" s="12" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="12" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="H5" s="12" t="str"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="12"/>
+      <x:c r="I5" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J5" s="30" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
-        <x:v>damageBoost</x:v>
+        <x:v>bbb</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>烈光</x:v>
+        <x:v>BBB</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>pickupDamage</x:v>
+        <x:v>pickupBBB</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>lightDamage</x:v>
+        <x:v>lightRadius</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>10</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F6" s="12" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G6" s="12" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="H6" s="12" t="str"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H6" s="12"/>
+      <x:c r="I6" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J6" s="30" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>defenseBoost</x:v>
+        <x:v>ppa</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>守護</x:v>
+        <x:v>PPA</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>pickupDefense</x:v>
+        <x:v>pickupPPA</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>damageReduction</x:v>
+        <x:v>healthDrainReduction</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>0.12</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="12" t="n">
         <x:v>0.5</x:v>
@@ -1523,33 +1629,23 @@
       <x:c r="G7" s="12" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H7" s="12" t="str"/>
+      <x:c r="H7" s="12"/>
+      <x:c r="I7" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="30" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="12" t="str">
-        <x:v>youthFruit</x:v>
-      </x:c>
-      <x:c r="B8" s="12" t="str">
-        <x:v>青春果</x:v>
-      </x:c>
-      <x:c r="C8" s="12" t="str">
-        <x:v>pickupAge</x:v>
-      </x:c>
-      <x:c r="D8" s="12" t="str">
-        <x:v>ageReduction</x:v>
-      </x:c>
-      <x:c r="E8" s="12" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F8" s="12" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G8" s="12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H8" s="12" t="n">
-        <x:v>35</x:v>
-      </x:c>
+      <x:c r="A8" s="12"/>
+      <x:c r="B8" s="12"/>
+      <x:c r="C8" s="12"/>
+      <x:c r="D8" s="12"/>
+      <x:c r="E8" s="12"/>
+      <x:c r="F8" s="12"/>
+      <x:c r="G8" s="12"/>
+      <x:c r="H8" s="12"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2595,16 +2691,16 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>pickupLight</x:v>
+        <x:v>pickupNNE</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>pickupLight</x:v>
+        <x:v>pickupNNE</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
         <x:v>assets/items/light-radius.png</x:v>
       </x:c>
-      <x:c r="D9" s="12" t="str"/>
-      <x:c r="E9" s="12" t="str"/>
+      <x:c r="D9" s="12"/>
+      <x:c r="E9" s="12"/>
       <x:c r="F9" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -2632,14 +2728,16 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
-        <x:v>pickupSpeed</x:v>
+        <x:v>pickupYSS</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>pickupSpeed</x:v>
-      </x:c>
-      <x:c r="C10" s="12" t="str"/>
-      <x:c r="D10" s="12" t="str"/>
-      <x:c r="E10" s="12" t="str"/>
+        <x:v>pickupYSS</x:v>
+      </x:c>
+      <x:c r="C10" s="12" t="str">
+        <x:v>assets/items/YSS.png</x:v>
+      </x:c>
+      <x:c r="D10" s="12"/>
+      <x:c r="E10" s="12"/>
       <x:c r="F10" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -2667,14 +2765,16 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>pickupDamage</x:v>
+        <x:v>pickupBBB</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>pickupDamage</x:v>
-      </x:c>
-      <x:c r="C11" s="12" t="str"/>
-      <x:c r="D11" s="12" t="str"/>
-      <x:c r="E11" s="12" t="str"/>
+        <x:v>pickupBBB</x:v>
+      </x:c>
+      <x:c r="C11" s="12" t="str">
+        <x:v>assets/items/BBB.png</x:v>
+      </x:c>
+      <x:c r="D11" s="12"/>
+      <x:c r="E11" s="12"/>
       <x:c r="F11" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -2702,14 +2802,16 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>pickupDefense</x:v>
+        <x:v>pickupPPA</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>pickupDefense</x:v>
-      </x:c>
-      <x:c r="C12" s="12" t="str"/>
-      <x:c r="D12" s="12" t="str"/>
-      <x:c r="E12" s="12" t="str"/>
+        <x:v>pickupPPA</x:v>
+      </x:c>
+      <x:c r="C12" s="12" t="str">
+        <x:v>assets/items/ppa-light-radius.png</x:v>
+      </x:c>
+      <x:c r="D12" s="12"/>
+      <x:c r="E12" s="12"/>
       <x:c r="F12" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -2723,10 +2825,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J12" s="12" t="str">
-        <x:v>rect</x:v>
+        <x:v>circle</x:v>
       </x:c>
       <x:c r="K12" s="12" t="n">
-        <x:v>5617407</x:v>
+        <x:v>11958503</x:v>
       </x:c>
       <x:c r="L12" s="12" t="n">
         <x:v>24</x:v>
@@ -2736,39 +2838,19 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="12" t="str">
-        <x:v>pickupAge</x:v>
-      </x:c>
-      <x:c r="B13" s="12" t="str">
-        <x:v>pickupAge</x:v>
-      </x:c>
-      <x:c r="C13" s="12" t="str"/>
-      <x:c r="D13" s="12" t="str"/>
-      <x:c r="E13" s="12" t="str"/>
-      <x:c r="F13" s="12" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G13" s="12" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="H13" s="12" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="I13" s="12" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J13" s="12" t="str">
-        <x:v>circle</x:v>
-      </x:c>
-      <x:c r="K13" s="12" t="n">
-        <x:v>11958503</x:v>
-      </x:c>
-      <x:c r="L13" s="12" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="M13" s="12" t="n">
-        <x:v>24</x:v>
-      </x:c>
+      <x:c r="A13" s="12"/>
+      <x:c r="B13" s="12"/>
+      <x:c r="C13" s="12"/>
+      <x:c r="D13" s="12"/>
+      <x:c r="E13" s="12"/>
+      <x:c r="F13" s="12"/>
+      <x:c r="G13" s="12"/>
+      <x:c r="H13" s="12"/>
+      <x:c r="I13" s="12"/>
+      <x:c r="J13" s="12"/>
+      <x:c r="K13" s="12"/>
+      <x:c r="L13" s="12"/>
+      <x:c r="M13" s="12"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>